<commit_message>
Update du .gitignore et du BOM. Ajout des traces pour le cristal,port usb mini etconnecteur pour le moteur.
</commit_message>
<xml_diff>
--- a/Projet Yawgmoth - BOM.xlsx
+++ b/Projet Yawgmoth - BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\H26\Projet fin de DEC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\H26\Projet-Yawgmoth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00F7C794-E8FA-4B64-8222-981876A5A158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA5879D9-63F0-4DD7-83FD-C9CB336A15D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15870" yWindow="360" windowWidth="15990" windowHeight="24720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="40">
   <si>
     <t>Item #</t>
   </si>
@@ -62,9 +62,6 @@
     <t>SMT32F103</t>
   </si>
   <si>
-    <t>N20</t>
-  </si>
-  <si>
     <t>Supplier 1</t>
   </si>
   <si>
@@ -144,6 +141,18 @@
   </si>
   <si>
     <t>STM32F103CBT6</t>
+  </si>
+  <si>
+    <t>LTS-4802BJR-H1</t>
+  </si>
+  <si>
+    <t>Affichage 7 segments LED verte</t>
+  </si>
+  <si>
+    <t>port mini usb</t>
+  </si>
+  <si>
+    <t>Adafruit motor</t>
   </si>
 </sst>
 </file>
@@ -562,16 +571,16 @@
         <v>6</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="L1" s="1" t="s">
         <v>7</v>
@@ -585,13 +594,13 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2">
         <v>8.43</v>
@@ -601,16 +610,16 @@
         <v>8.43</v>
       </c>
       <c r="H2" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s">
         <v>35</v>
       </c>
-      <c r="I2" t="s">
-        <v>36</v>
-      </c>
       <c r="J2" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2" t="s">
         <v>16</v>
-      </c>
-      <c r="K2" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -618,23 +627,23 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D3">
         <v>1</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G3">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -642,23 +651,23 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J4" t="s">
         <v>15</v>
-      </c>
-      <c r="G4">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -666,23 +675,23 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D5">
         <v>1</v>
       </c>
       <c r="E5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J5" t="s">
         <v>15</v>
-      </c>
-      <c r="G5">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -690,20 +699,20 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
         <v>23</v>
       </c>
-      <c r="C6" t="s">
-        <v>24</v>
-      </c>
       <c r="E6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J6" t="s">
         <v>15</v>
-      </c>
-      <c r="G6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J6" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -711,16 +720,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F7">
         <v>2.4500000000000002</v>
@@ -730,13 +739,13 @@
         <v>4.9000000000000004</v>
       </c>
       <c r="J7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="L7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -744,16 +753,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D8">
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F8">
         <v>3.28</v>
@@ -763,45 +772,60 @@
         <v>3.28</v>
       </c>
       <c r="J8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="K8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
       <c r="D9">
         <v>1</v>
       </c>
       <c r="E9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F9">
+        <v>0.87</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>0.87</v>
+      </c>
+      <c r="J9" t="s">
         <v>15</v>
       </c>
-      <c r="G9">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="J9" t="s">
-        <v>16</v>
-      </c>
       <c r="K9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
+      <c r="C10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G10">
         <f t="shared" si="0"/>
@@ -813,7 +837,7 @@
         <v>10</v>
       </c>
       <c r="E11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G11">
         <f>D11*F11</f>
@@ -825,7 +849,7 @@
         <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G12">
         <f t="shared" si="0"/>
@@ -837,7 +861,7 @@
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G13">
         <f t="shared" si="0"/>
@@ -849,7 +873,7 @@
         <v>13</v>
       </c>
       <c r="E14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
@@ -861,7 +885,7 @@
         <v>14</v>
       </c>
       <c r="E15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G15">
         <f t="shared" si="0"/>
@@ -873,7 +897,7 @@
         <v>15</v>
       </c>
       <c r="E16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G16">
         <f t="shared" si="0"/>
@@ -885,7 +909,7 @@
         <v>16</v>
       </c>
       <c r="E17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G17">
         <f t="shared" si="0"/>
@@ -897,7 +921,7 @@
         <v>17</v>
       </c>
       <c r="E18" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G18">
         <f t="shared" si="0"/>
@@ -909,7 +933,7 @@
         <v>18</v>
       </c>
       <c r="E19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G19">
         <f t="shared" si="0"/>
@@ -921,7 +945,7 @@
         <v>19</v>
       </c>
       <c r="E20" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G20">
         <f t="shared" si="0"/>
@@ -933,7 +957,7 @@
         <v>20</v>
       </c>
       <c r="E21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G21">
         <f t="shared" si="0"/>
@@ -945,7 +969,7 @@
         <v>21</v>
       </c>
       <c r="E22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G22">
         <f t="shared" si="0"/>

</xml_diff>